<commit_message>
randomness update and cleaning
</commit_message>
<xml_diff>
--- a/Output/phase2_significance_results_2026-04-15.xlsx
+++ b/Output/phase2_significance_results_2026-04-15.xlsx
@@ -532,16 +532,16 @@
         <v>16720</v>
       </c>
       <c r="E2" t="n">
-        <v>0.028</v>
+        <v>0.0291</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0333</v>
+        <v>0.0346</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0052</v>
+        <v>0.0055</v>
       </c>
       <c r="H2" t="n">
-        <v>0.0024</v>
+        <v>0.0016</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -549,16 +549,16 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.805</v>
+        <v>0.8280999999999999</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9229000000000001</v>
+        <v>0.9752</v>
       </c>
       <c r="L2" t="n">
-        <v>0.1179</v>
+        <v>0.1471</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0486</v>
+        <v>0.0236</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -566,18 +566,22 @@
         </is>
       </c>
       <c r="O2" t="n">
-        <v>0.4928</v>
+        <v>0.506</v>
       </c>
       <c r="P2" t="n">
-        <v>0.5583</v>
+        <v>0.5905</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0655</v>
+        <v>0.08450000000000001</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0713</v>
-      </c>
-      <c r="S2" t="inlineStr"/>
+        <v>0.0343</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -597,39 +601,39 @@
         <v>16848</v>
       </c>
       <c r="E3" t="n">
-        <v>0.026</v>
+        <v>0.0266</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0272</v>
+        <v>0.0281</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0013</v>
+        <v>0.0016</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2268</v>
+        <v>0.1821</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
-        <v>0.8332000000000001</v>
+        <v>0.8535</v>
       </c>
       <c r="K3" t="n">
-        <v>0.7869</v>
+        <v>0.8142</v>
       </c>
       <c r="L3" t="n">
-        <v>-0.0463</v>
+        <v>-0.0392</v>
       </c>
       <c r="M3" t="n">
         <v>1</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>0.513</v>
+        <v>0.5245</v>
       </c>
       <c r="P3" t="n">
-        <v>0.4714</v>
+        <v>0.4902</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.0415</v>
+        <v>-0.0343</v>
       </c>
       <c r="R3" t="n">
         <v>1</v>
@@ -765,39 +769,39 @@
         <v>2401</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0262</v>
+        <v>0.0273</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0308</v>
+        <v>0.0317</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0047</v>
+        <v>0.0043</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1605</v>
+        <v>0.1808</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
-        <v>1.0368</v>
+        <v>1.0752</v>
       </c>
       <c r="K2" t="n">
-        <v>0.9121</v>
+        <v>0.9278</v>
       </c>
       <c r="L2" t="n">
-        <v>-0.1247</v>
+        <v>-0.1475</v>
       </c>
       <c r="M2" t="n">
         <v>1</v>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="n">
-        <v>0.669</v>
+        <v>0.6889</v>
       </c>
       <c r="P2" t="n">
-        <v>0.5337</v>
+        <v>0.5427999999999999</v>
       </c>
       <c r="Q2" t="n">
-        <v>-0.1353</v>
+        <v>-0.1462</v>
       </c>
       <c r="R2" t="n">
         <v>1</v>
@@ -822,42 +826,42 @@
         <v>2445</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0269</v>
+        <v>0.0273</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0307</v>
+        <v>0.0315</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0038</v>
+        <v>0.0042</v>
       </c>
       <c r="H3" t="n">
-        <v>0.2088</v>
+        <v>0.1853</v>
       </c>
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="n">
-        <v>0.8545</v>
+        <v>0.8527</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8824</v>
+        <v>0.8929</v>
       </c>
       <c r="L3" t="n">
-        <v>0.028</v>
+        <v>0.0401</v>
       </c>
       <c r="M3" t="n">
-        <v>0.4384</v>
+        <v>0.4121</v>
       </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="n">
-        <v>0.5353</v>
+        <v>0.5341</v>
       </c>
       <c r="P3" t="n">
-        <v>0.5296</v>
+        <v>0.5368000000000001</v>
       </c>
       <c r="Q3" t="n">
-        <v>-0.0057</v>
+        <v>0.0027</v>
       </c>
       <c r="R3" t="n">
-        <v>1</v>
+        <v>0.4907</v>
       </c>
       <c r="S3" t="inlineStr"/>
     </row>
@@ -869,49 +873,49 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BNLX_ChurnP_10eu_test_export.csv</t>
+          <t>BNLX_ChurnP_10_test_export.csv</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2594</v>
+        <v>2593</v>
       </c>
       <c r="D4" t="n">
-        <v>2379</v>
+        <v>2349</v>
       </c>
       <c r="E4" t="n">
-        <v>0.0235</v>
+        <v>0.0305</v>
       </c>
       <c r="F4" t="n">
-        <v>0.0252</v>
+        <v>0.0341</v>
       </c>
       <c r="G4" t="n">
-        <v>0.0017</v>
+        <v>0.0036</v>
       </c>
       <c r="H4" t="n">
-        <v>0.3484</v>
+        <v>0.2376</v>
       </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="n">
-        <v>0.7973</v>
+        <v>0.9903999999999999</v>
       </c>
       <c r="K4" t="n">
-        <v>0.6781</v>
+        <v>1.0377</v>
       </c>
       <c r="L4" t="n">
-        <v>-0.1192</v>
+        <v>0.0473</v>
       </c>
       <c r="M4" t="n">
-        <v>1</v>
+        <v>0.4142</v>
       </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="n">
-        <v>0.4751</v>
+        <v>0.5881999999999999</v>
       </c>
       <c r="P4" t="n">
-        <v>0.4227</v>
+        <v>0.5837</v>
       </c>
       <c r="Q4" t="n">
-        <v>-0.0524</v>
+        <v>-0.0045</v>
       </c>
       <c r="R4" t="n">
         <v>1</v>
@@ -926,49 +930,49 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BNLX_ChurnP_10_test_export.csv</t>
+          <t>BNLX_ChurnP_10eu_test_export.csv</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2593</v>
+        <v>2594</v>
       </c>
       <c r="D5" t="n">
-        <v>2349</v>
+        <v>2379</v>
       </c>
       <c r="E5" t="n">
-        <v>0.0305</v>
+        <v>0.0247</v>
       </c>
       <c r="F5" t="n">
-        <v>0.0324</v>
+        <v>0.0261</v>
       </c>
       <c r="G5" t="n">
-        <v>0.0019</v>
+        <v>0.0014</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3519</v>
+        <v>0.3778</v>
       </c>
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="n">
-        <v>0.9903999999999999</v>
+        <v>0.8573</v>
       </c>
       <c r="K5" t="n">
-        <v>1.0014</v>
+        <v>0.6926</v>
       </c>
       <c r="L5" t="n">
-        <v>0.0109</v>
+        <v>-0.1647</v>
       </c>
       <c r="M5" t="n">
-        <v>0.4799</v>
+        <v>1</v>
       </c>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="n">
-        <v>0.5881999999999999</v>
+        <v>0.5096000000000001</v>
       </c>
       <c r="P5" t="n">
-        <v>0.556</v>
+        <v>0.4277</v>
       </c>
       <c r="Q5" t="n">
-        <v>-0.0323</v>
+        <v>-0.0819</v>
       </c>
       <c r="R5" t="n">
         <v>1</v>
@@ -993,42 +997,42 @@
         <v>2406</v>
       </c>
       <c r="E6" t="n">
-        <v>0.0235</v>
+        <v>0.0242</v>
       </c>
       <c r="F6" t="n">
         <v>0.0249</v>
       </c>
       <c r="G6" t="n">
-        <v>0.0015</v>
+        <v>0.0007</v>
       </c>
       <c r="H6" t="n">
-        <v>0.3678</v>
+        <v>0.4359</v>
       </c>
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="n">
-        <v>0.7272</v>
+        <v>0.7562</v>
       </c>
       <c r="K6" t="n">
         <v>0.8599</v>
       </c>
       <c r="L6" t="n">
-        <v>0.1327</v>
+        <v>0.1037</v>
       </c>
       <c r="M6" t="n">
-        <v>0.2487</v>
+        <v>0.2988</v>
       </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="n">
-        <v>0.4463</v>
+        <v>0.462</v>
       </c>
       <c r="P6" t="n">
         <v>0.5115</v>
       </c>
       <c r="Q6" t="n">
-        <v>0.06519999999999999</v>
+        <v>0.0495</v>
       </c>
       <c r="R6" t="n">
-        <v>0.2919</v>
+        <v>0.3394</v>
       </c>
       <c r="S6" t="inlineStr"/>
     </row>
@@ -1053,10 +1057,10 @@
         <v>0.0227</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0192</v>
+        <v>0.02</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.0035</v>
+        <v>-0.0027</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
@@ -1066,10 +1070,10 @@
         <v>0.6589</v>
       </c>
       <c r="K7" t="n">
-        <v>0.5434</v>
+        <v>0.6137</v>
       </c>
       <c r="L7" t="n">
-        <v>-0.1154</v>
+        <v>-0.0452</v>
       </c>
       <c r="M7" t="n">
         <v>1</v>
@@ -1079,13 +1083,13 @@
         <v>0.388</v>
       </c>
       <c r="P7" t="n">
-        <v>0.354</v>
+        <v>0.4033</v>
       </c>
       <c r="Q7" t="n">
-        <v>-0.0341</v>
+        <v>0.0152</v>
       </c>
       <c r="R7" t="n">
-        <v>1</v>
+        <v>0.444</v>
       </c>
       <c r="S7" t="inlineStr"/>
     </row>
@@ -1107,39 +1111,39 @@
         <v>2372</v>
       </c>
       <c r="E8" t="n">
-        <v>0.0285</v>
+        <v>0.0293</v>
       </c>
       <c r="F8" t="n">
-        <v>0.0278</v>
+        <v>0.0291</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.0007</v>
+        <v>-0.0002</v>
       </c>
       <c r="H8" t="n">
         <v>1</v>
       </c>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="n">
-        <v>0.7695</v>
+        <v>0.7861</v>
       </c>
       <c r="K8" t="n">
-        <v>0.6405999999999999</v>
+        <v>0.6838</v>
       </c>
       <c r="L8" t="n">
-        <v>-0.1288</v>
+        <v>-0.1022</v>
       </c>
       <c r="M8" t="n">
         <v>1</v>
       </c>
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="n">
-        <v>0.4895</v>
+        <v>0.5017</v>
       </c>
       <c r="P8" t="n">
-        <v>0.3965</v>
+        <v>0.4287</v>
       </c>
       <c r="Q8" t="n">
-        <v>-0.093</v>
+        <v>-0.07290000000000001</v>
       </c>
       <c r="R8" t="n">
         <v>1</v>
@@ -1164,16 +1168,16 @@
         <v>2685</v>
       </c>
       <c r="E9" t="n">
-        <v>0.0262</v>
+        <v>0.0272</v>
       </c>
       <c r="F9" t="n">
-        <v>0.0369</v>
+        <v>0.038</v>
       </c>
       <c r="G9" t="n">
-        <v>0.0107</v>
+        <v>0.0108</v>
       </c>
       <c r="H9" t="n">
-        <v>0.0112</v>
+        <v>0.0117</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1181,16 +1185,16 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.765</v>
+        <v>0.7949000000000001</v>
       </c>
       <c r="K9" t="n">
-        <v>1.0774</v>
+        <v>1.1006</v>
       </c>
       <c r="L9" t="n">
-        <v>0.3124</v>
+        <v>0.3057</v>
       </c>
       <c r="M9" t="n">
-        <v>0.042</v>
+        <v>0.0476</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1198,16 +1202,16 @@
         </is>
       </c>
       <c r="O9" t="n">
-        <v>0.4712</v>
+        <v>0.4863</v>
       </c>
       <c r="P9" t="n">
-        <v>0.6514</v>
+        <v>0.6646</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.1802</v>
+        <v>0.1783</v>
       </c>
       <c r="R9" t="n">
-        <v>0.0566</v>
+        <v>0.06</v>
       </c>
       <c r="S9" t="inlineStr"/>
     </row>
@@ -1219,52 +1223,56 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BNLX_ChurnP_5eu_test_export.csv</t>
+          <t>BNLX_ChurnP_10_test_export.csv</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>3044</v>
+        <v>2274</v>
       </c>
       <c r="D10" t="n">
-        <v>2711</v>
+        <v>2065</v>
       </c>
       <c r="E10" t="n">
-        <v>0.0246</v>
+        <v>0.0303</v>
       </c>
       <c r="F10" t="n">
-        <v>0.0317</v>
+        <v>0.0397</v>
       </c>
       <c r="G10" t="n">
-        <v>0.0071</v>
+        <v>0.0094</v>
       </c>
       <c r="H10" t="n">
-        <v>0.0523</v>
-      </c>
-      <c r="I10" t="inlineStr"/>
+        <v>0.0468</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
       <c r="J10" t="n">
-        <v>0.5872000000000001</v>
+        <v>1.064</v>
       </c>
       <c r="K10" t="n">
-        <v>0.787</v>
+        <v>1.2511</v>
       </c>
       <c r="L10" t="n">
-        <v>0.1998</v>
+        <v>0.1871</v>
       </c>
       <c r="M10" t="n">
-        <v>0.0738</v>
+        <v>0.2485</v>
       </c>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="n">
-        <v>0.3554</v>
+        <v>0.6172</v>
       </c>
       <c r="P10" t="n">
-        <v>0.4949</v>
+        <v>0.7169</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.1395</v>
+        <v>0.0997</v>
       </c>
       <c r="R10" t="n">
-        <v>0.061</v>
+        <v>0.2662</v>
       </c>
       <c r="S10" t="inlineStr"/>
     </row>
@@ -1286,42 +1294,42 @@
         <v>2116</v>
       </c>
       <c r="E11" t="n">
-        <v>0.0267</v>
+        <v>0.0286</v>
       </c>
       <c r="F11" t="n">
-        <v>0.035</v>
+        <v>0.0364</v>
       </c>
       <c r="G11" t="n">
-        <v>0.0083</v>
+        <v>0.0078</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0594</v>
+        <v>0.07439999999999999</v>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="n">
-        <v>0.7358</v>
+        <v>0.775</v>
       </c>
       <c r="K11" t="n">
-        <v>1.0529</v>
+        <v>1.0756</v>
       </c>
       <c r="L11" t="n">
-        <v>0.3171</v>
+        <v>0.3005</v>
       </c>
       <c r="M11" t="n">
-        <v>0.0781</v>
+        <v>0.09080000000000001</v>
       </c>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="n">
-        <v>0.492</v>
+        <v>0.5149</v>
       </c>
       <c r="P11" t="n">
-        <v>0.6388</v>
+        <v>0.6563</v>
       </c>
       <c r="Q11" t="n">
-        <v>0.1468</v>
+        <v>0.1414</v>
       </c>
       <c r="R11" t="n">
-        <v>0.1652</v>
+        <v>0.1755</v>
       </c>
       <c r="S11" t="inlineStr"/>
     </row>
@@ -1333,52 +1341,52 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BNLX_ChurnP_10_test_export.csv</t>
+          <t>BNLX_ChurnP_5eu_test_export.csv</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2274</v>
+        <v>3044</v>
       </c>
       <c r="D12" t="n">
-        <v>2065</v>
+        <v>2711</v>
       </c>
       <c r="E12" t="n">
-        <v>0.029</v>
+        <v>0.026</v>
       </c>
       <c r="F12" t="n">
-        <v>0.0368</v>
+        <v>0.0321</v>
       </c>
       <c r="G12" t="n">
-        <v>0.0078</v>
+        <v>0.0061</v>
       </c>
       <c r="H12" t="n">
-        <v>0.0756</v>
+        <v>0.0828</v>
       </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="n">
-        <v>1.0283</v>
+        <v>0.6274999999999999</v>
       </c>
       <c r="K12" t="n">
-        <v>1.0686</v>
+        <v>0.8195</v>
       </c>
       <c r="L12" t="n">
-        <v>0.0403</v>
+        <v>0.192</v>
       </c>
       <c r="M12" t="n">
-        <v>0.4317</v>
+        <v>0.09</v>
       </c>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="n">
-        <v>0.5954</v>
+        <v>0.3797</v>
       </c>
       <c r="P12" t="n">
-        <v>0.6071</v>
+        <v>0.5185</v>
       </c>
       <c r="Q12" t="n">
-        <v>0.0117</v>
+        <v>0.1388</v>
       </c>
       <c r="R12" t="n">
-        <v>0.4656</v>
+        <v>0.0697</v>
       </c>
       <c r="S12" t="inlineStr"/>
     </row>
@@ -1400,42 +1408,42 @@
         <v>2373</v>
       </c>
       <c r="E13" t="n">
-        <v>0.0296</v>
+        <v>0.03</v>
       </c>
       <c r="F13" t="n">
-        <v>0.0341</v>
+        <v>0.0354</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0045</v>
+        <v>0.0054</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1801</v>
+        <v>0.1395</v>
       </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="n">
-        <v>0.7985</v>
+        <v>0.8004</v>
       </c>
       <c r="K13" t="n">
-        <v>0.9615</v>
+        <v>0.9991</v>
       </c>
       <c r="L13" t="n">
-        <v>0.163</v>
+        <v>0.1987</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1686</v>
+        <v>0.1236</v>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="n">
-        <v>0.4889</v>
+        <v>0.49</v>
       </c>
       <c r="P13" t="n">
-        <v>0.6187</v>
+        <v>0.644</v>
       </c>
       <c r="Q13" t="n">
-        <v>0.1298</v>
+        <v>0.154</v>
       </c>
       <c r="R13" t="n">
-        <v>0.1194</v>
+        <v>0.0839</v>
       </c>
       <c r="S13" t="inlineStr"/>
     </row>
@@ -1457,42 +1465,42 @@
         <v>2526</v>
       </c>
       <c r="E14" t="n">
-        <v>0.0281</v>
+        <v>0.0292</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0285</v>
+        <v>0.0297</v>
       </c>
       <c r="G14" t="n">
         <v>0.0004</v>
       </c>
       <c r="H14" t="n">
-        <v>0.4656</v>
+        <v>0.4622</v>
       </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="n">
-        <v>0.7622</v>
+        <v>0.768</v>
       </c>
       <c r="K14" t="n">
-        <v>0.8596</v>
+        <v>0.9098000000000001</v>
       </c>
       <c r="L14" t="n">
-        <v>0.0974</v>
+        <v>0.1418</v>
       </c>
       <c r="M14" t="n">
-        <v>0.3057</v>
+        <v>0.2338</v>
       </c>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="n">
-        <v>0.469</v>
+        <v>0.4689</v>
       </c>
       <c r="P14" t="n">
-        <v>0.4967</v>
+        <v>0.5225</v>
       </c>
       <c r="Q14" t="n">
-        <v>0.0278</v>
+        <v>0.0536</v>
       </c>
       <c r="R14" t="n">
-        <v>0.4084</v>
+        <v>0.3298</v>
       </c>
       <c r="S14" t="inlineStr"/>
     </row>
@@ -1514,39 +1522,39 @@
         <v>2244</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0329</v>
+        <v>0.0333</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0303</v>
+        <v>0.0321</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.0026</v>
+        <v>-0.0012</v>
       </c>
       <c r="H15" t="n">
         <v>1</v>
       </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="n">
-        <v>1.0297</v>
+        <v>1.0398</v>
       </c>
       <c r="K15" t="n">
-        <v>0.6758999999999999</v>
+        <v>0.7134</v>
       </c>
       <c r="L15" t="n">
-        <v>-0.3538</v>
+        <v>-0.3264</v>
       </c>
       <c r="M15" t="n">
         <v>1</v>
       </c>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="n">
-        <v>0.6244</v>
+        <v>0.6326000000000001</v>
       </c>
       <c r="P15" t="n">
-        <v>0.4083</v>
+        <v>0.4308</v>
       </c>
       <c r="Q15" t="n">
-        <v>-0.2161</v>
+        <v>-0.2019</v>
       </c>
       <c r="R15" t="n">
         <v>1</v>

</xml_diff>